<commit_message>
Replace original xlsx with styled version
</commit_message>
<xml_diff>
--- a/top_candidates.xlsx
+++ b/top_candidates.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$D$101</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +27,49 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007D45E0"/>
+        <bgColor rgb="007D45E0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F8FAFC"/>
+        <bgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFD700"/>
+        <bgColor rgb="00FFD700"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +77,50 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00E2E8F0"/>
+      </left>
+      <right style="thin">
+        <color rgb="00E2E8F0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00E2E8F0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00E2E8F0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -415,1830 +488,1837 @@
   </sheetPr>
   <dimension ref="A1:D101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="120" customWidth="1" min="4" max="4"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>candidate_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>rank</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>score</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>reasoning</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>CAND_0087630</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Current Role: AI Engineer at Vedantu with 7.2 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Elasticsearch, Embeddings, OpenSearch) matching the JD. Platform Signals: Based in Gurgaon (willing to relocate); 30-day notice (highly immediate availability); active GitHub (score 23).</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>CAND_0091072</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="6" t="n">
         <v>0.9751</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Paytm with 7.9 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Vector Search) matching the JD. Platform Signals: Based in Indore; 30-day notice (highly immediate availability).</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>CAND_0074123</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="8" t="n">
         <v>0.9197</v>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>Current Role: Data Scientist at CRED with 6.9 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (pgvector, NLP, ETL) matching the JD. Platform Signals: Based in Bhubaneswar (willing to relocate); 30-day notice (highly immediate availability).</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>CAND_0097567</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="6" t="n">
         <v>4</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="6" t="n">
         <v>0.892</v>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at PharmEasy with 6.3 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Computer Vision, REST APIs, Data Science) matching the JD. Platform Signals: Based in Bangalore (willing to relocate); 60-day notice.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>CAND_0033445</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="8" t="n">
         <v>5</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="8" t="n">
         <v>0.8754</v>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>Current Role: ML Engineer at Vedantu with 6.8 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Deep Learning, Agile, Information Retrieval) matching the JD. Platform Signals: Based in Ahmedabad; 30-day notice (highly immediate availability).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="5" t="inlineStr">
         <is>
           <t>CAND_0054409</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="6" t="n">
         <v>6</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="6" t="n">
         <v>0.8421999999999999</v>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Current Role: Data Engineer at Freshworks with 7.4 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Qdrant) matching the JD. Platform Signals: Based in Mumbai; 30-day notice (highly immediate availability).</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>CAND_0079387</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="8" t="n">
         <v>7</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8" s="8" t="n">
         <v>0.7785</v>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
         <is>
           <t>Current Role: AI Engineer at Microsoft with 6.9 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Vector Search, OpenSearch) matching the JD. Platform Signals: Based in Trivandrum; 30-day notice (highly immediate availability); strong GitHub portfolio (score 64).</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
+      <c r="A9" s="5" t="inlineStr">
         <is>
           <t>CAND_0032216</t>
         </is>
       </c>
-      <c r="B9" t="n">
+      <c r="B9" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9" s="6" t="n">
         <v>0.7675</v>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>Current Role: ML Engineer at upGrad with 6.1 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Qdrant, Vector Search) matching the JD. Platform Signals: Based in Chennai (willing to relocate); 30-day notice (highly immediate availability); active GitHub (score 14).</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>CAND_0081846</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="8" t="n">
         <v>9</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10" s="8" t="n">
         <v>0.7343</v>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>Current Role: Lead AI Engineer at Razorpay with 6.7 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Elasticsearch, Vector Search, Embeddings) matching the JD. Platform Signals: Based in Jaipur (willing to relocate); 30-day notice (highly immediate availability); active GitHub (score 33).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>CAND_0098288</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="6" t="n">
         <v>10</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11" s="6" t="n">
         <v>0.7287</v>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>Current Role: Junior ML Engineer at Vedantu with 6.7 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (RAG) matching the JD. Platform Signals: Based in Mumbai (willing to relocate); 60-day notice; active GitHub (score 30).</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>CAND_0080051</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" s="8" t="n">
         <v>11</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12" s="8" t="n">
         <v>0.7066</v>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>Current Role: Data Scientist at Niramai with 5.2 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Feature Engineering, NLP, Information Retrieval) matching the JD. Platform Signals: Based in Gurgaon; 30-day notice (highly immediate availability); active GitHub (score 34).</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
         <is>
           <t>CAND_0066710</t>
         </is>
       </c>
-      <c r="B13" t="n">
+      <c r="B13" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C13" s="6" t="n">
         <v>0.6955</v>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>Current Role: Data Engineer at Vedantu with 6.9 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (ASR, Go, QLoRA) matching the JD. Platform Signals: Based in Trivandrum (willing to relocate); 30-day notice (highly immediate availability); active GitHub (score 37).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>CAND_0029100</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="B14" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C14" s="8" t="n">
         <v>0.6927</v>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="D14" s="7" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Paytm with 7.9 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Airflow, Time Series, Deep Learning) matching the JD. Platform Signals: Based in Gurgaon; 30-day notice (highly immediate availability); active GitHub (score 50).</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="5" t="inlineStr">
         <is>
           <t>CAND_0087506</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="B15" s="6" t="n">
         <v>14</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C15" s="6" t="n">
         <v>0.6927</v>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Vedantu with 7.4 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Time Series, AWS, TypeScript) matching the JD. Platform Signals: Based in Kolkata; 30-day notice (highly immediate availability).</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>CAND_0021884</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B16" s="8" t="n">
         <v>15</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C16" s="8" t="n">
         <v>0.6844</v>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="7" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Razorpay with 7.7 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Kubernetes, Redux, Microservices) matching the JD. Platform Signals: Based in Bhubaneswar; 30-day notice (highly immediate availability); active GitHub (score 30).</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>CAND_0004300</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" s="6" t="n">
         <v>16</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C17" s="6" t="n">
         <v>0.6761</v>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="5" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at PharmEasy with 7.4 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (OpenSearch) matching the JD. Platform Signals: Based in Indore; 60-day notice.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>CAND_0007052</t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="B18" s="8" t="n">
         <v>17</v>
       </c>
-      <c r="C18" t="n">
+      <c r="C18" s="8" t="n">
         <v>0.6706</v>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="7" t="inlineStr">
         <is>
           <t>Current Role: ML Engineer at Unacademy with 6.5 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (RAG, Weaviate, Milvus) matching the JD. Platform Signals: Based in Pune (direct hybrid match); 60-day notice.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr">
         <is>
           <t>CAND_0095023</t>
         </is>
       </c>
-      <c r="B19" t="n">
+      <c r="B19" s="6" t="n">
         <v>18</v>
       </c>
-      <c r="C19" t="n">
+      <c r="C19" s="6" t="n">
         <v>0.6651</v>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at CRED with 7.8 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (PowerPoint, Kubernetes, QLoRA) matching the JD. Platform Signals: Based in Mumbai; 60-day notice.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>CAND_0007994</t>
         </is>
       </c>
-      <c r="B20" t="n">
+      <c r="B20" s="8" t="n">
         <v>19</v>
       </c>
-      <c r="C20" t="n">
+      <c r="C20" s="8" t="n">
         <v>0.6512</v>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D20" s="7" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Razorpay with 6.6 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Milvus) matching the JD. Platform Signals: Based in Mumbai; 60-day notice.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="5" t="inlineStr">
         <is>
           <t>CAND_0079984</t>
         </is>
       </c>
-      <c r="B21" t="n">
+      <c r="B21" s="6" t="n">
         <v>20</v>
       </c>
-      <c r="C21" t="n">
+      <c r="C21" s="6" t="n">
         <v>0.6512</v>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Pied Piper with 6.6 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Computer Vision, Agile, GraphQL) matching the JD. Platform Signals: Based in Gurgaon; 60-day notice; active GitHub (score 58).</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>CAND_0089464</t>
         </is>
       </c>
-      <c r="B22" t="n">
+      <c r="B22" s="8" t="n">
         <v>21</v>
       </c>
-      <c r="C22" t="n">
+      <c r="C22" s="8" t="n">
         <v>0.6429</v>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="7" t="inlineStr">
         <is>
           <t>Current Role: Data Engineer at Zoho with 6.1 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Weaviate) matching the JD. Platform Signals: Based in Noida (direct hybrid match); 90-day notice; strong GitHub portfolio (score 62).</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="5" t="inlineStr">
         <is>
           <t>CAND_0018539</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="B23" s="6" t="n">
         <v>22</v>
       </c>
-      <c r="C23" t="n">
+      <c r="C23" s="6" t="n">
         <v>0.6346000000000001</v>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Pied Piper with 7.6 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Project Management, Microservices, Recommendation Systems) matching the JD. Platform Signals: Based in Mumbai; 60-day notice; active GitHub (score 52).</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>CAND_0093193</t>
         </is>
       </c>
-      <c r="B24" t="n">
+      <c r="B24" s="8" t="n">
         <v>23</v>
       </c>
-      <c r="C24" t="n">
+      <c r="C24" s="8" t="n">
         <v>0.6346000000000001</v>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D24" s="7" t="inlineStr">
         <is>
           <t>Current Role: Senior Machine Learning Engineer at Niramai with 7.9 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Qdrant, OpenSearch) matching the JD. Platform Signals: Based in Bangalore; 45-day notice; active GitHub (score 34).</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="5" t="inlineStr">
         <is>
           <t>CAND_0024890</t>
         </is>
       </c>
-      <c r="B25" t="n">
+      <c r="B25" s="6" t="n">
         <v>24</v>
       </c>
-      <c r="C25" t="n">
+      <c r="C25" s="6" t="n">
         <v>0.6318</v>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>Current Role: Data Engineer at Hooli with 6.9 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Weaviate) matching the JD. Platform Signals: Based in Chandigarh (willing to relocate); 60-day notice.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="7" t="inlineStr">
         <is>
           <t>CAND_0074465</t>
         </is>
       </c>
-      <c r="B26" t="n">
+      <c r="B26" s="8" t="n">
         <v>25</v>
       </c>
-      <c r="C26" t="n">
+      <c r="C26" s="8" t="n">
         <v>0.6318</v>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D26" s="7" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Razorpay with 7.1 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (RAG) matching the JD. Platform Signals: Based in Pune (direct hybrid match); 90-day notice; active GitHub (score 32).</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="5" t="inlineStr">
         <is>
           <t>CAND_0006693</t>
         </is>
       </c>
-      <c r="B27" t="n">
+      <c r="B27" s="6" t="n">
         <v>26</v>
       </c>
-      <c r="C27" t="n">
+      <c r="C27" s="6" t="n">
         <v>0.6152</v>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr">
         <is>
           <t>Current Role: Data Engineer at BYJU'S with 6.4 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Forecasting, MLOps, TensorFlow) matching the JD. Platform Signals: Based in Hyderabad; 60-day notice; active GitHub (score 38).</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="7" t="inlineStr">
         <is>
           <t>CAND_0099641</t>
         </is>
       </c>
-      <c r="B28" t="n">
+      <c r="B28" s="8" t="n">
         <v>27</v>
       </c>
-      <c r="C28" t="n">
+      <c r="C28" s="8" t="n">
         <v>0.6152</v>
       </c>
-      <c r="D28" t="inlineStr">
+      <c r="D28" s="7" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at CRED with 6.9 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (dbt, Deep Learning, Airflow) matching the JD. Platform Signals: Based in Gurgaon; 120-day notice; active GitHub (score 6).</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" t="inlineStr">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>CAND_0014988</t>
         </is>
       </c>
-      <c r="B29" t="n">
+      <c r="B29" s="6" t="n">
         <v>28</v>
       </c>
-      <c r="C29" t="n">
+      <c r="C29" s="6" t="n">
         <v>0.5654</v>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D29" s="5" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Hooli with 7.9 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Microservices, GCP, React) matching the JD. Platform Signals: Based in Bangalore; 60-day notice; active GitHub (score 33).</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="7" t="inlineStr">
         <is>
           <t>CAND_0041772</t>
         </is>
       </c>
-      <c r="B30" t="n">
+      <c r="B30" s="8" t="n">
         <v>29</v>
       </c>
-      <c r="C30" t="n">
+      <c r="C30" s="8" t="n">
         <v>0.5571</v>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D30" s="7" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at BYJU'S with 6.0 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Angular, Docker, ASR) matching the JD. Platform Signals: Based in Gurgaon; 90-day notice.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>CAND_0015493</t>
         </is>
       </c>
-      <c r="B31" t="n">
+      <c r="B31" s="6" t="n">
         <v>30</v>
       </c>
-      <c r="C31" t="n">
+      <c r="C31" s="6" t="n">
         <v>0.5488</v>
       </c>
-      <c r="D31" t="inlineStr">
+      <c r="D31" s="5" t="inlineStr">
         <is>
           <t>Current Role: Data Scientist at CRED with 6.4 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (gRPC, scikit-learn, Semantic Search) matching the JD. Platform Signals: Based in Vizag; 30-day notice (highly immediate availability); strong GitHub portfolio (score 65).</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" t="inlineStr">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>CAND_0077337</t>
         </is>
       </c>
-      <c r="B32" t="n">
+      <c r="B32" s="8" t="n">
         <v>31</v>
       </c>
-      <c r="C32" t="n">
+      <c r="C32" s="8" t="n">
         <v>0.5433</v>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D32" s="7" t="inlineStr">
         <is>
           <t>Current Role: Staff Machine Learning Engineer at Paytm with 7.0 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Pinecone, RAG, Qdrant) matching the JD. Platform Signals: Based in Kochi (willing to relocate); 60-day notice; strong GitHub portfolio (score 68).</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="A33" s="5" t="inlineStr">
         <is>
           <t>CAND_0082086</t>
         </is>
       </c>
-      <c r="B33" t="n">
+      <c r="B33" s="6" t="n">
         <v>32</v>
       </c>
-      <c r="C33" t="n">
+      <c r="C33" s="6" t="n">
         <v>0.5294</v>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D33" s="5" t="inlineStr">
         <is>
           <t>Current Role: Senior Software Engineer (ML) at Razorpay with 6.0 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (FAISS, Pinecone, Milvus) matching the JD. Platform Signals: Based in Delhi; 45-day notice; strong GitHub portfolio (score 82).</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
+      <c r="A34" s="7" t="inlineStr">
         <is>
           <t>CAND_0058688</t>
         </is>
       </c>
-      <c r="B34" t="n">
+      <c r="B34" s="8" t="n">
         <v>33</v>
       </c>
-      <c r="C34" t="n">
+      <c r="C34" s="8" t="n">
         <v>0.5266</v>
       </c>
-      <c r="D34" t="inlineStr">
+      <c r="D34" s="7" t="inlineStr">
         <is>
           <t>Current Role: AI Engineer at Vedantu with 6.7 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Embeddings, Milvus) matching the JD. Platform Signals: Based in Berlin (willing to relocate); 15-day notice (highly immediate availability); active GitHub (score 39).</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>CAND_0073645</t>
         </is>
       </c>
-      <c r="B35" t="n">
+      <c r="B35" s="6" t="n">
         <v>34</v>
       </c>
-      <c r="C35" t="n">
+      <c r="C35" s="6" t="n">
         <v>0.5266</v>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D35" s="5" t="inlineStr">
         <is>
           <t>Current Role: Data Engineer at Vedantu with 6.7 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Forecasting, Speech Recognition, Reinforcement Learning) matching the JD. Platform Signals: Based in Delhi; 90-day notice; active GitHub (score 38).</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
+      <c r="A36" s="7" t="inlineStr">
         <is>
           <t>CAND_0008049</t>
         </is>
       </c>
-      <c r="B36" t="n">
+      <c r="B36" s="8" t="n">
         <v>35</v>
       </c>
-      <c r="C36" t="n">
+      <c r="C36" s="8" t="n">
         <v>0.5155999999999999</v>
       </c>
-      <c r="D36" t="inlineStr">
+      <c r="D36" s="7" t="inlineStr">
         <is>
           <t>Current Role: ML Engineer at Niramai with 6.3 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (RAG) matching the JD. Platform Signals: Based in Pune (direct hybrid match); 60-day notice; active GitHub (score 58).</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>CAND_0058463</t>
         </is>
       </c>
-      <c r="B37" t="n">
+      <c r="B37" s="6" t="n">
         <v>36</v>
       </c>
-      <c r="C37" t="n">
+      <c r="C37" s="6" t="n">
         <v>0.5155999999999999</v>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D37" s="5" t="inlineStr">
         <is>
           <t>Current Role: Senior Software Engineer at Zoho with 7.5 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Pinecone) matching the JD. Platform Signals: Based in Kolkata (willing to relocate); 30-day notice (highly immediate availability).</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" t="inlineStr">
+      <c r="A38" s="7" t="inlineStr">
         <is>
           <t>CAND_0096440</t>
         </is>
       </c>
-      <c r="B38" t="n">
+      <c r="B38" s="8" t="n">
         <v>37</v>
       </c>
-      <c r="C38" t="n">
+      <c r="C38" s="8" t="n">
         <v>0.4934</v>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D38" s="7" t="inlineStr">
         <is>
           <t>Current Role: Data Engineer at Razorpay with 7.7 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Kafka, Time Series, Speech Recognition) matching the JD. Platform Signals: Based in Hyderabad; 90-day notice; active GitHub (score 29).</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" t="inlineStr">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>CAND_0071941</t>
         </is>
       </c>
-      <c r="B39" t="n">
+      <c r="B39" s="6" t="n">
         <v>38</v>
       </c>
-      <c r="C39" t="n">
+      <c r="C39" s="6" t="n">
         <v>0.4768</v>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="5" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Razorpay with 5.2 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (FastAPI, Redux, PostgreSQL) matching the JD. Platform Signals: Based in Noida (direct hybrid match); 30-day notice (highly immediate availability).</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="inlineStr">
+      <c r="A40" s="7" t="inlineStr">
         <is>
           <t>CAND_0079468</t>
         </is>
       </c>
-      <c r="B40" t="n">
+      <c r="B40" s="8" t="n">
         <v>39</v>
       </c>
-      <c r="C40" t="n">
+      <c r="C40" s="8" t="n">
         <v>0.4768</v>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="7" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Razorpay with 5.8 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Reinforcement Learning, Agile, Data Science) matching the JD. Platform Signals: Based in Pune (direct hybrid match); 30-day notice (highly immediate availability).</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>CAND_0051532</t>
         </is>
       </c>
-      <c r="B41" t="n">
+      <c r="B41" s="6" t="n">
         <v>40</v>
       </c>
-      <c r="C41" t="n">
+      <c r="C41" s="6" t="n">
         <v>0.474</v>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="5" t="inlineStr">
         <is>
           <t>Current Role: Data Engineer at Razorpay with 7.0 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (MLOps, Computer Vision, Forecasting) matching the JD. Platform Signals: Based in Jaipur; 30-day notice (highly immediate availability).</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="inlineStr">
+      <c r="A42" s="7" t="inlineStr">
         <is>
           <t>CAND_0019724</t>
         </is>
       </c>
-      <c r="B42" t="n">
+      <c r="B42" s="8" t="n">
         <v>41</v>
       </c>
-      <c r="C42" t="n">
+      <c r="C42" s="8" t="n">
         <v>0.4713</v>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="7" t="inlineStr">
         <is>
           <t>Current Role: Data Engineer at Freshworks with 7.7 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (MLOps, Azure, Redux) matching the JD. Platform Signals: Based in Pune (direct hybrid match); 60-day notice; active GitHub (score 41).</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="inlineStr">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>CAND_0068811</t>
         </is>
       </c>
-      <c r="B43" t="n">
+      <c r="B43" s="6" t="n">
         <v>42</v>
       </c>
-      <c r="C43" t="n">
+      <c r="C43" s="6" t="n">
         <v>0.4574</v>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="5" t="inlineStr">
         <is>
           <t>Current Role: Applied ML Engineer at Freshworks with 8.0 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Vector Search, Qdrant, Embeddings) matching the JD. Platform Signals: Based in Pune (direct hybrid match); 30-day notice (highly immediate availability); active GitHub (score 23).</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="inlineStr">
+      <c r="A44" s="7" t="inlineStr">
         <is>
           <t>CAND_0050398</t>
         </is>
       </c>
-      <c r="B44" t="n">
+      <c r="B44" s="8" t="n">
         <v>43</v>
       </c>
-      <c r="C44" t="n">
+      <c r="C44" s="8" t="n">
         <v>0.4547</v>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="7" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at upGrad with 7.7 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (RAG) matching the JD. Platform Signals: Based in Vizag; 90-day notice.</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="inlineStr">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>CAND_0091424</t>
         </is>
       </c>
-      <c r="B45" t="n">
+      <c r="B45" s="6" t="n">
         <v>44</v>
       </c>
-      <c r="C45" t="n">
+      <c r="C45" s="6" t="n">
         <v>0.4491</v>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="5" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at CRED with 6.3 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Data Science, Semantic Search, PowerPoint) matching the JD. Platform Signals: Based in Gurgaon (willing to relocate); 90-day notice.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
+      <c r="A46" s="7" t="inlineStr">
         <is>
           <t>CAND_0068273</t>
         </is>
       </c>
-      <c r="B46" t="n">
+      <c r="B46" s="8" t="n">
         <v>45</v>
       </c>
-      <c r="C46" t="n">
+      <c r="C46" s="8" t="n">
         <v>0.4464</v>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="7" t="inlineStr">
         <is>
           <t>Current Role: Data Scientist at Wysa with 6.6 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (pgvector, Deep Learning, ASR) matching the JD. Platform Signals: Based in Pune (direct hybrid match); 45-day notice.</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
+      <c r="A47" s="5" t="inlineStr">
         <is>
           <t>CAND_0080766</t>
         </is>
       </c>
-      <c r="B47" t="n">
+      <c r="B47" s="6" t="n">
         <v>46</v>
       </c>
-      <c r="C47" t="n">
+      <c r="C47" s="6" t="n">
         <v>0.4436</v>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="5" t="inlineStr">
         <is>
           <t>Current Role: Staff Machine Learning Engineer at Salesforce with 8.8 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Elasticsearch, OpenSearch, Milvus) matching the JD. Platform Signals: Based in Coimbatore (willing to relocate); 90-day notice; active GitHub (score 32).</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
+      <c r="A48" s="7" t="inlineStr">
         <is>
           <t>CAND_0054940</t>
         </is>
       </c>
-      <c r="B48" t="n">
+      <c r="B48" s="8" t="n">
         <v>47</v>
       </c>
-      <c r="C48" t="n">
+      <c r="C48" s="8" t="n">
         <v>0.4408</v>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="7" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Razorpay with 7.7 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Redis, Deep Learning, gRPC) matching the JD. Platform Signals: Based in Gurgaon; 90-day notice.</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="inlineStr">
+      <c r="A49" s="5" t="inlineStr">
         <is>
           <t>CAND_0007412</t>
         </is>
       </c>
-      <c r="B49" t="n">
+      <c r="B49" s="6" t="n">
         <v>48</v>
       </c>
-      <c r="C49" t="n">
+      <c r="C49" s="6" t="n">
         <v>0.4381</v>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49" s="5" t="inlineStr">
         <is>
           <t>Current Role: Applied ML Engineer at Zoho with 7.4 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Pinecone, Milvus, RAG) matching the JD. Platform Signals: Based in Noida (direct hybrid match); 120-day notice; active GitHub (score 36).</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
+      <c r="A50" s="7" t="inlineStr">
         <is>
           <t>CAND_0044063</t>
         </is>
       </c>
-      <c r="B50" t="n">
+      <c r="B50" s="8" t="n">
         <v>49</v>
       </c>
-      <c r="C50" t="n">
+      <c r="C50" s="8" t="n">
         <v>0.4325</v>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D50" s="7" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Initech with 7.8 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (ASR, NLP, Microservices) matching the JD. Platform Signals: Based in Bhubaneswar; 60-day notice.</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="5" t="inlineStr">
         <is>
           <t>CAND_0034787</t>
         </is>
       </c>
-      <c r="B51" t="n">
+      <c r="B51" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="C51" t="n">
+      <c r="C51" s="6" t="n">
         <v>0.427</v>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D51" s="5" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at PhonePe with 6.3 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Go, dbt, Reinforcement Learning) matching the JD. Platform Signals: Based in Noida (direct hybrid match); 30-day notice (highly immediate availability); strong GitHub portfolio (score 60).</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="7" t="inlineStr">
         <is>
           <t>CAND_0020350</t>
         </is>
       </c>
-      <c r="B52" t="n">
+      <c r="B52" s="8" t="n">
         <v>51</v>
       </c>
-      <c r="C52" t="n">
+      <c r="C52" s="8" t="n">
         <v>0.4242</v>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D52" s="7" t="inlineStr">
         <is>
           <t>Current Role: AI Engineer at Zoho with 5.8 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (FAISS, Vector Search) matching the JD. Platform Signals: Based in Jaipur; 30-day notice (highly immediate availability).</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="5" t="inlineStr">
         <is>
           <t>CAND_0018320</t>
         </is>
       </c>
-      <c r="B53" t="n">
+      <c r="B53" s="6" t="n">
         <v>52</v>
       </c>
-      <c r="C53" t="n">
+      <c r="C53" s="6" t="n">
         <v>0.4187</v>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D53" s="5" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at CRED with 7.0 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (FAISS) matching the JD. Platform Signals: Based in New York (willing to relocate); 90-day notice; strong GitHub portfolio (score 66).</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="7" t="inlineStr">
         <is>
           <t>CAND_0086735</t>
         </is>
       </c>
-      <c r="B54" t="n">
+      <c r="B54" s="8" t="n">
         <v>53</v>
       </c>
-      <c r="C54" t="n">
+      <c r="C54" s="8" t="n">
         <v>0.4159</v>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D54" s="7" t="inlineStr">
         <is>
           <t>Current Role: Data Engineer at PharmEasy with 5.6 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (FastAPI, ASR, Speech Recognition) matching the JD. Platform Signals: Based in Gurgaon; 30-day notice (highly immediate availability).</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" s="5" t="inlineStr">
         <is>
           <t>CAND_0098438</t>
         </is>
       </c>
-      <c r="B55" t="n">
+      <c r="B55" s="6" t="n">
         <v>54</v>
       </c>
-      <c r="C55" t="n">
+      <c r="C55" s="6" t="n">
         <v>0.4131</v>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D55" s="5" t="inlineStr">
         <is>
           <t>Current Role: Data Engineer at Freshworks with 6.4 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (RAG, Elasticsearch) matching the JD. Platform Signals: Based in Pune (direct hybrid match); 60-day notice.</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="7" t="inlineStr">
         <is>
           <t>CAND_0083701</t>
         </is>
       </c>
-      <c r="B56" t="n">
+      <c r="B56" s="8" t="n">
         <v>55</v>
       </c>
-      <c r="C56" t="n">
+      <c r="C56" s="8" t="n">
         <v>0.4104</v>
       </c>
-      <c r="D56" t="inlineStr">
+      <c r="D56" s="7" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Razorpay with 7.7 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Milvus) matching the JD. Platform Signals: Based in Noida (direct hybrid match); 120-day notice; active GitHub (score 38).</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
+      <c r="A57" s="5" t="inlineStr">
         <is>
           <t>CAND_0087796</t>
         </is>
       </c>
-      <c r="B57" t="n">
+      <c r="B57" s="6" t="n">
         <v>56</v>
       </c>
-      <c r="C57" t="n">
+      <c r="C57" s="6" t="n">
         <v>0.4021</v>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D57" s="5" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Pied Piper with 6.3 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Speech Recognition, MLOps, Angular) matching the JD. Platform Signals: Based in Jaipur (willing to relocate); 90-day notice; active GitHub (score 34).</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
+      <c r="A58" s="7" t="inlineStr">
         <is>
           <t>CAND_0072688</t>
         </is>
       </c>
-      <c r="B58" t="n">
+      <c r="B58" s="8" t="n">
         <v>57</v>
       </c>
-      <c r="C58" t="n">
+      <c r="C58" s="8" t="n">
         <v>0.391</v>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="D58" s="7" t="inlineStr">
         <is>
           <t>Current Role: Data Scientist at Niramai with 6.9 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Milvus, Qdrant) matching the JD. Platform Signals: Based in Pune (direct hybrid match); 45-day notice; active GitHub (score 11).</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
+      <c r="A59" s="5" t="inlineStr">
         <is>
           <t>CAND_0033350</t>
         </is>
       </c>
-      <c r="B59" t="n">
+      <c r="B59" s="6" t="n">
         <v>58</v>
       </c>
-      <c r="C59" t="n">
+      <c r="C59" s="6" t="n">
         <v>0.3772</v>
       </c>
-      <c r="D59" t="inlineStr">
+      <c r="D59" s="5" t="inlineStr">
         <is>
           <t>Current Role: Data Scientist at upGrad with 6.2 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (OpenSearch) matching the JD. Platform Signals: Based in Coimbatore; 90-day notice.</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="inlineStr">
+      <c r="A60" s="7" t="inlineStr">
         <is>
           <t>CAND_0020017</t>
         </is>
       </c>
-      <c r="B60" t="n">
+      <c r="B60" s="8" t="n">
         <v>59</v>
       </c>
-      <c r="C60" t="n">
+      <c r="C60" s="8" t="n">
         <v>0.3689</v>
       </c>
-      <c r="D60" t="inlineStr">
+      <c r="D60" s="7" t="inlineStr">
         <is>
           <t>Current Role: Senior Software Engineer at Unacademy with 7.0 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Machine Learning, Time Series, REST APIs) matching the JD. Platform Signals: Based in Bangalore; 30-day notice (highly immediate availability); active GitHub (score 54).</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="inlineStr">
+      <c r="A61" s="5" t="inlineStr">
         <is>
           <t>CAND_0076959</t>
         </is>
       </c>
-      <c r="B61" t="n">
+      <c r="B61" s="6" t="n">
         <v>60</v>
       </c>
-      <c r="C61" t="n">
+      <c r="C61" s="6" t="n">
         <v>0.3689</v>
       </c>
-      <c r="D61" t="inlineStr">
+      <c r="D61" s="5" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Zoho with 7.6 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (OpenSearch) matching the JD. Platform Signals: Based in Austin (willing to relocate); 60-day notice; strong GitHub portfolio (score 65).</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" s="7" t="inlineStr">
         <is>
           <t>CAND_0017771</t>
         </is>
       </c>
-      <c r="B62" t="n">
+      <c r="B62" s="8" t="n">
         <v>61</v>
       </c>
-      <c r="C62" t="n">
+      <c r="C62" s="8" t="n">
         <v>0.3661</v>
       </c>
-      <c r="D62" t="inlineStr">
+      <c r="D62" s="7" t="inlineStr">
         <is>
           <t>Current Role: Senior Software Engineer at Unacademy with 7.8 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Computer Vision, Information Retrieval, Azure) matching the JD. Platform Signals: Based in Noida (direct hybrid match); 60-day notice; active GitHub (score 54).</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="inlineStr">
+      <c r="A63" s="5" t="inlineStr">
         <is>
           <t>CAND_0002995</t>
         </is>
       </c>
-      <c r="B63" t="n">
+      <c r="B63" s="6" t="n">
         <v>62</v>
       </c>
-      <c r="C63" t="n">
+      <c r="C63" s="6" t="n">
         <v>0.3633</v>
       </c>
-      <c r="D63" t="inlineStr">
+      <c r="D63" s="5" t="inlineStr">
         <is>
           <t>Current Role: Senior Software Engineer at Hooli with 7.9 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Qdrant) matching the JD. Platform Signals: Based in Pune (direct hybrid match); 60-day notice.</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" t="inlineStr">
+      <c r="A64" s="7" t="inlineStr">
         <is>
           <t>CAND_0083910</t>
         </is>
       </c>
-      <c r="B64" t="n">
+      <c r="B64" s="8" t="n">
         <v>63</v>
       </c>
-      <c r="C64" t="n">
+      <c r="C64" s="8" t="n">
         <v>0.3522</v>
       </c>
-      <c r="D64" t="inlineStr">
+      <c r="D64" s="7" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at CRED with 5.1 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Redux, Terraform, Semantic Search) matching the JD. Platform Signals: Based in Mumbai; 30-day notice (highly immediate availability); active GitHub (score 41).</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" t="inlineStr">
+      <c r="A65" s="5" t="inlineStr">
         <is>
           <t>CAND_0005277</t>
         </is>
       </c>
-      <c r="B65" t="n">
+      <c r="B65" s="6" t="n">
         <v>64</v>
       </c>
-      <c r="C65" t="n">
+      <c r="C65" s="6" t="n">
         <v>0.3495</v>
       </c>
-      <c r="D65" t="inlineStr">
+      <c r="D65" s="5" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at CRED with 6.1 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Computer Vision, Redis, NLP) matching the JD. Platform Signals: Based in Ahmedabad (willing to relocate); 90-day notice.</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
+      <c r="A66" s="7" t="inlineStr">
         <is>
           <t>CAND_0084928</t>
         </is>
       </c>
-      <c r="B66" t="n">
+      <c r="B66" s="8" t="n">
         <v>65</v>
       </c>
-      <c r="C66" t="n">
+      <c r="C66" s="8" t="n">
         <v>0.3495</v>
       </c>
-      <c r="D66" t="inlineStr">
+      <c r="D66" s="7" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Hooli with 6.1 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Microservices, GraphQL, Azure) matching the JD. Platform Signals: Based in Delhi; 90-day notice.</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
+      <c r="A67" s="5" t="inlineStr">
         <is>
           <t>CAND_0032914</t>
         </is>
       </c>
-      <c r="B67" t="n">
+      <c r="B67" s="6" t="n">
         <v>66</v>
       </c>
-      <c r="C67" t="n">
+      <c r="C67" s="6" t="n">
         <v>0.3439</v>
       </c>
-      <c r="D67" t="inlineStr">
+      <c r="D67" s="5" t="inlineStr">
         <is>
           <t>Current Role: Senior Data Engineer at Razorpay with 7.6 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Feature Engineering, NLP, Speech Recognition) matching the JD. Platform Signals: Based in Gurgaon; 60-day notice.</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" t="inlineStr">
+      <c r="A68" s="7" t="inlineStr">
         <is>
           <t>CAND_0097443</t>
         </is>
       </c>
-      <c r="B68" t="n">
+      <c r="B68" s="8" t="n">
         <v>67</v>
       </c>
-      <c r="C68" t="n">
+      <c r="C68" s="8" t="n">
         <v>0.3356</v>
       </c>
-      <c r="D68" t="inlineStr">
+      <c r="D68" s="7" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Hooli with 6.6 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (FastAPI, React, scikit-learn) matching the JD. Platform Signals: Based in Bhubaneswar (willing to relocate); 150-day notice.</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" t="inlineStr">
+      <c r="A69" s="5" t="inlineStr">
         <is>
           <t>CAND_0066944</t>
         </is>
       </c>
-      <c r="B69" t="n">
+      <c r="B69" s="6" t="n">
         <v>68</v>
       </c>
-      <c r="C69" t="n">
+      <c r="C69" s="6" t="n">
         <v>0.3329</v>
       </c>
-      <c r="D69" t="inlineStr">
+      <c r="D69" s="5" t="inlineStr">
         <is>
           <t>Current Role: Data Engineer at Vedantu with 7.0 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Pinecone, Vector Search) matching the JD. Platform Signals: Based in Ahmedabad; 90-day notice; strong GitHub portfolio (score 62).</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr">
+      <c r="A70" s="7" t="inlineStr">
         <is>
           <t>CAND_0022478</t>
         </is>
       </c>
-      <c r="B70" t="n">
+      <c r="B70" s="8" t="n">
         <v>69</v>
       </c>
-      <c r="C70" t="n">
+      <c r="C70" s="8" t="n">
         <v>0.3135</v>
       </c>
-      <c r="D70" t="inlineStr">
+      <c r="D70" s="7" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at BYJU'S with 7.0 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (OpenSearch) matching the JD. Platform Signals: Based in Bangalore (willing to relocate); 90-day notice; strong GitHub portfolio (score 60).</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
+      <c r="A71" s="5" t="inlineStr">
         <is>
           <t>CAND_0044091</t>
         </is>
       </c>
-      <c r="B71" t="n">
+      <c r="B71" s="6" t="n">
         <v>70</v>
       </c>
-      <c r="C71" t="n">
+      <c r="C71" s="6" t="n">
         <v>0.3135</v>
       </c>
-      <c r="D71" t="inlineStr">
+      <c r="D71" s="5" t="inlineStr">
         <is>
           <t>Current Role: ML Engineer at Vedantu with 6.5 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (FAISS) matching the JD. Platform Signals: Based in Indore; 120-day notice; active GitHub (score 28).</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" t="inlineStr">
+      <c r="A72" s="7" t="inlineStr">
         <is>
           <t>CAND_0066258</t>
         </is>
       </c>
-      <c r="B72" t="n">
+      <c r="B72" s="8" t="n">
         <v>71</v>
       </c>
-      <c r="C72" t="n">
+      <c r="C72" s="8" t="n">
         <v>0.308</v>
       </c>
-      <c r="D72" t="inlineStr">
+      <c r="D72" s="7" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Initech with 7.0 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (OpenSearch) matching the JD. Platform Signals: Based in Indore; 30-day notice (highly immediate availability).</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" t="inlineStr">
+      <c r="A73" s="5" t="inlineStr">
         <is>
           <t>CAND_0052428</t>
         </is>
       </c>
-      <c r="B73" t="n">
+      <c r="B73" s="6" t="n">
         <v>72</v>
       </c>
-      <c r="C73" t="n">
+      <c r="C73" s="6" t="n">
         <v>0.3052</v>
       </c>
-      <c r="D73" t="inlineStr">
+      <c r="D73" s="5" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at CRED with 6.2 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (OpenSearch) matching the JD. Platform Signals: Based in Ahmedabad (willing to relocate); 60-day notice.</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" t="inlineStr">
+      <c r="A74" s="7" t="inlineStr">
         <is>
           <t>CAND_0046575</t>
         </is>
       </c>
-      <c r="B74" t="n">
+      <c r="B74" s="8" t="n">
         <v>73</v>
       </c>
-      <c r="C74" t="n">
+      <c r="C74" s="8" t="n">
         <v>0.3024</v>
       </c>
-      <c r="D74" t="inlineStr">
+      <c r="D74" s="7" t="inlineStr">
         <is>
           <t>Current Role: Data Engineer at Pied Piper with 7.1 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Weaviate) matching the JD. Platform Signals: Based in Chandigarh; 60-day notice.</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" t="inlineStr">
+      <c r="A75" s="5" t="inlineStr">
         <is>
           <t>CAND_0056210</t>
         </is>
       </c>
-      <c r="B75" t="n">
+      <c r="B75" s="6" t="n">
         <v>74</v>
       </c>
-      <c r="C75" t="n">
+      <c r="C75" s="6" t="n">
         <v>0.2997</v>
       </c>
-      <c r="D75" t="inlineStr">
+      <c r="D75" s="5" t="inlineStr">
         <is>
           <t>Current Role: Data Engineer at BYJU'S with 6.7 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (OpenSearch) matching the JD. Platform Signals: Based in Bangalore; 90-day notice; active GitHub (score 29).</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr">
+      <c r="A76" s="7" t="inlineStr">
         <is>
           <t>CAND_0098846</t>
         </is>
       </c>
-      <c r="B76" t="n">
+      <c r="B76" s="8" t="n">
         <v>75</v>
       </c>
-      <c r="C76" t="n">
+      <c r="C76" s="8" t="n">
         <v>0.2997</v>
       </c>
-      <c r="D76" t="inlineStr">
+      <c r="D76" s="7" t="inlineStr">
         <is>
           <t>Current Role: AI Engineer at upGrad with 7.6 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Qdrant) matching the JD. Platform Signals: Based in Indore (willing to relocate); 45-day notice; strong GitHub portfolio (score 86).</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
+      <c r="A77" s="5" t="inlineStr">
         <is>
           <t>CAND_0072660</t>
         </is>
       </c>
-      <c r="B77" t="n">
+      <c r="B77" s="6" t="n">
         <v>76</v>
       </c>
-      <c r="C77" t="n">
+      <c r="C77" s="6" t="n">
         <v>0.2969</v>
       </c>
-      <c r="D77" t="inlineStr">
+      <c r="D77" s="5" t="inlineStr">
         <is>
           <t>Current Role: Machine Learning Engineer at Unacademy with 7.1 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (OpenSearch, FAISS, Elasticsearch) matching the JD. Platform Signals: Based in Berlin; 30-day notice (highly immediate availability).</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" t="inlineStr">
+      <c r="A78" s="7" t="inlineStr">
         <is>
           <t>CAND_0001912</t>
         </is>
       </c>
-      <c r="B78" t="n">
+      <c r="B78" s="8" t="n">
         <v>77</v>
       </c>
-      <c r="C78" t="n">
+      <c r="C78" s="8" t="n">
         <v>0.2886</v>
       </c>
-      <c r="D78" t="inlineStr">
+      <c r="D78" s="7" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Razorpay with 6.7 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Computer Vision, Terraform, dbt) matching the JD. Platform Signals: Based in Mumbai (willing to relocate); 60-day notice.</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr">
+      <c r="A79" s="5" t="inlineStr">
         <is>
           <t>CAND_0088711</t>
         </is>
       </c>
-      <c r="B79" t="n">
+      <c r="B79" s="6" t="n">
         <v>78</v>
       </c>
-      <c r="C79" t="n">
+      <c r="C79" s="6" t="n">
         <v>0.2886</v>
       </c>
-      <c r="D79" t="inlineStr">
+      <c r="D79" s="5" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Hooli with 8.4 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Scrum, Microservices, Machine Learning) matching the JD. Platform Signals: Based in Mumbai; 60-day notice; active GitHub (score 4).</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" t="inlineStr">
+      <c r="A80" s="7" t="inlineStr">
         <is>
           <t>CAND_0063645</t>
         </is>
       </c>
-      <c r="B80" t="n">
+      <c r="B80" s="8" t="n">
         <v>79</v>
       </c>
-      <c r="C80" t="n">
+      <c r="C80" s="8" t="n">
         <v>0.2858</v>
       </c>
-      <c r="D80" t="inlineStr">
+      <c r="D80" s="7" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Vedantu with 7.8 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Spring Boot, MLOps, Time Series) matching the JD. Platform Signals: Based in Mumbai; 120-day notice; strong GitHub portfolio (score 72).</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" t="inlineStr">
+      <c r="A81" s="5" t="inlineStr">
         <is>
           <t>CAND_0018293</t>
         </is>
       </c>
-      <c r="B81" t="n">
+      <c r="B81" s="6" t="n">
         <v>80</v>
       </c>
-      <c r="C81" t="n">
+      <c r="C81" s="6" t="n">
         <v>0.2747</v>
       </c>
-      <c r="D81" t="inlineStr">
+      <c r="D81" s="5" t="inlineStr">
         <is>
           <t>Current Role: Data Scientist at PharmEasy with 5.6 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Weaviate) matching the JD. Platform Signals: Based in Indore (willing to relocate); 60-day notice.</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" t="inlineStr">
+      <c r="A82" s="7" t="inlineStr">
         <is>
           <t>CAND_0091580</t>
         </is>
       </c>
-      <c r="B82" t="n">
+      <c r="B82" s="8" t="n">
         <v>81</v>
       </c>
-      <c r="C82" t="n">
+      <c r="C82" s="8" t="n">
         <v>0.2747</v>
       </c>
-      <c r="D82" t="inlineStr">
+      <c r="D82" s="7" t="inlineStr">
         <is>
           <t>Current Role: Data Scientist at Niramai with 5.5 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (FAISS, Qdrant) matching the JD. Platform Signals: Based in Noida (direct hybrid match); 60-day notice; strong GitHub portfolio (score 83).</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" t="inlineStr">
+      <c r="A83" s="5" t="inlineStr">
         <is>
           <t>CAND_0051630</t>
         </is>
       </c>
-      <c r="B83" t="n">
+      <c r="B83" s="6" t="n">
         <v>82</v>
       </c>
-      <c r="C83" t="n">
+      <c r="C83" s="6" t="n">
         <v>0.272</v>
       </c>
-      <c r="D83" t="inlineStr">
+      <c r="D83" s="5" t="inlineStr">
         <is>
           <t>Current Role: Machine Learning Engineer at Razorpay with 6.0 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Elasticsearch, Embeddings, OpenSearch) matching the JD. Platform Signals: Based in Kolkata; 90-day notice; strong GitHub portfolio (score 66).</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" t="inlineStr">
+      <c r="A84" s="7" t="inlineStr">
         <is>
           <t>CAND_0086818</t>
         </is>
       </c>
-      <c r="B84" t="n">
+      <c r="B84" s="8" t="n">
         <v>83</v>
       </c>
-      <c r="C84" t="n">
+      <c r="C84" s="8" t="n">
         <v>0.272</v>
       </c>
-      <c r="D84" t="inlineStr">
+      <c r="D84" s="7" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Hooli with 5.2 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Prompt Engineering, Marketing, ASR) matching the JD. Platform Signals: Based in Hyderabad (willing to relocate); 90-day notice; strong GitHub portfolio (score 61).</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" t="inlineStr">
+      <c r="A85" s="5" t="inlineStr">
         <is>
           <t>CAND_0015967</t>
         </is>
       </c>
-      <c r="B85" t="n">
+      <c r="B85" s="6" t="n">
         <v>84</v>
       </c>
-      <c r="C85" t="n">
+      <c r="C85" s="6" t="n">
         <v>0.2692</v>
       </c>
-      <c r="D85" t="inlineStr">
+      <c r="D85" s="5" t="inlineStr">
         <is>
           <t>Current Role: Senior Software Engineer (ML) at Razorpay with 5.4 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Pinecone, Embeddings) matching the JD. Platform Signals: Based in Hyderabad (willing to relocate); 30-day notice (highly immediate availability); active GitHub (score 26).</t>
         </is>
       </c>
     </row>
     <row r="86">
-      <c r="A86" t="inlineStr">
+      <c r="A86" s="7" t="inlineStr">
         <is>
           <t>CAND_0049116</t>
         </is>
       </c>
-      <c r="B86" t="n">
+      <c r="B86" s="8" t="n">
         <v>85</v>
       </c>
-      <c r="C86" t="n">
+      <c r="C86" s="8" t="n">
         <v>0.2692</v>
       </c>
-      <c r="D86" t="inlineStr">
+      <c r="D86" s="7" t="inlineStr">
         <is>
           <t>Current Role: Senior Data Engineer at Freshworks with 7.7 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Forecasting, Reinforcement Learning, QLoRA) matching the JD. Platform Signals: Based in Hyderabad; 60-day notice; active GitHub (score 13).</t>
         </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" t="inlineStr">
+      <c r="A87" s="5" t="inlineStr">
         <is>
           <t>CAND_0000665</t>
         </is>
       </c>
-      <c r="B87" t="n">
+      <c r="B87" s="6" t="n">
         <v>86</v>
       </c>
-      <c r="C87" t="n">
+      <c r="C87" s="6" t="n">
         <v>0.2637</v>
       </c>
-      <c r="D87" t="inlineStr">
+      <c r="D87" s="5" t="inlineStr">
         <is>
           <t>Current Role: Senior Software Engineer at PharmEasy with 6.2 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Embeddings) matching the JD. Platform Signals: Based in Pune (direct hybrid match); 90-day notice; active GitHub (score 57).</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" t="inlineStr">
+      <c r="A88" s="7" t="inlineStr">
         <is>
           <t>CAND_0040616</t>
         </is>
       </c>
-      <c r="B88" t="n">
+      <c r="B88" s="8" t="n">
         <v>87</v>
       </c>
-      <c r="C88" t="n">
+      <c r="C88" s="8" t="n">
         <v>0.2637</v>
       </c>
-      <c r="D88" t="inlineStr">
+      <c r="D88" s="7" t="inlineStr">
         <is>
           <t>Current Role: Senior Software Engineer at CRED with 6.8 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Data Science, Hadoop, TypeScript) matching the JD. Platform Signals: Based in Kochi; 30-day notice (highly immediate availability).</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" t="inlineStr">
+      <c r="A89" s="5" t="inlineStr">
         <is>
           <t>CAND_0065327</t>
         </is>
       </c>
-      <c r="B89" t="n">
+      <c r="B89" s="6" t="n">
         <v>88</v>
       </c>
-      <c r="C89" t="n">
+      <c r="C89" s="6" t="n">
         <v>0.2637</v>
       </c>
-      <c r="D89" t="inlineStr">
+      <c r="D89" s="5" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Pied Piper with 6.6 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Vector Search) matching the JD. Platform Signals: Based in Delhi; 120-day notice; strong GitHub portfolio (score 63).</t>
         </is>
       </c>
     </row>
     <row r="90">
-      <c r="A90" t="inlineStr">
+      <c r="A90" s="7" t="inlineStr">
         <is>
           <t>CAND_0010603</t>
         </is>
       </c>
-      <c r="B90" t="n">
+      <c r="B90" s="8" t="n">
         <v>89</v>
       </c>
-      <c r="C90" t="n">
+      <c r="C90" s="8" t="n">
         <v>0.2609</v>
       </c>
-      <c r="D90" t="inlineStr">
+      <c r="D90" s="7" t="inlineStr">
         <is>
           <t>Current Role: ML Engineer at BYJU'S with 5.3 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (OpenSearch) matching the JD. Platform Signals: Based in Bangalore; 90-day notice; strong GitHub portfolio (score 78).</t>
         </is>
       </c>
     </row>
     <row r="91">
-      <c r="A91" t="inlineStr">
+      <c r="A91" s="5" t="inlineStr">
         <is>
           <t>CAND_0020375</t>
         </is>
       </c>
-      <c r="B91" t="n">
+      <c r="B91" s="6" t="n">
         <v>90</v>
       </c>
-      <c r="C91" t="n">
+      <c r="C91" s="6" t="n">
         <v>0.2554</v>
       </c>
-      <c r="D91" t="inlineStr">
+      <c r="D91" s="5" t="inlineStr">
         <is>
           <t>Current Role: Data Engineer at Pied Piper with 5.4 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Forecasting, Marketing, NLP) matching the JD. Platform Signals: Based in Bangalore (willing to relocate); 90-day notice; active GitHub (score 58).</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" t="inlineStr">
+      <c r="A92" s="7" t="inlineStr">
         <is>
           <t>CAND_0007090</t>
         </is>
       </c>
-      <c r="B92" t="n">
+      <c r="B92" s="8" t="n">
         <v>91</v>
       </c>
-      <c r="C92" t="n">
+      <c r="C92" s="8" t="n">
         <v>0.2526</v>
       </c>
-      <c r="D92" t="inlineStr">
+      <c r="D92" s="7" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Zoho with 6.4 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Learning to Rank, ASR, Time Series) matching the JD. Platform Signals: Based in Hyderabad (willing to relocate); 60-day notice.</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" t="inlineStr">
+      <c r="A93" s="5" t="inlineStr">
         <is>
           <t>CAND_0099464</t>
         </is>
       </c>
-      <c r="B93" t="n">
+      <c r="B93" s="6" t="n">
         <v>92</v>
       </c>
-      <c r="C93" t="n">
+      <c r="C93" s="6" t="n">
         <v>0.2498</v>
       </c>
-      <c r="D93" t="inlineStr">
+      <c r="D93" s="5" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Initech with 8.0 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (GCP, Agile, JavaScript) matching the JD. Platform Signals: Based in Delhi; 90-day notice; strong GitHub portfolio (score 61).</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" t="inlineStr">
+      <c r="A94" s="7" t="inlineStr">
         <is>
           <t>CAND_0015097</t>
         </is>
       </c>
-      <c r="B94" t="n">
+      <c r="B94" s="8" t="n">
         <v>93</v>
       </c>
-      <c r="C94" t="n">
+      <c r="C94" s="8" t="n">
         <v>0.236</v>
       </c>
-      <c r="D94" t="inlineStr">
+      <c r="D94" s="7" t="inlineStr">
         <is>
           <t>Current Role: Senior Software Engineer (ML) at Zoho with 6.0 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Speech Recognition, BigQuery, Python) matching the JD. Platform Signals: Based in Coimbatore; 30-day notice (highly immediate availability); active GitHub (score 21).</t>
         </is>
       </c>
     </row>
     <row r="95">
-      <c r="A95" t="inlineStr">
+      <c r="A95" s="5" t="inlineStr">
         <is>
           <t>CAND_0050215</t>
         </is>
       </c>
-      <c r="B95" t="n">
+      <c r="B95" s="6" t="n">
         <v>94</v>
       </c>
-      <c r="C95" t="n">
+      <c r="C95" s="6" t="n">
         <v>0.236</v>
       </c>
-      <c r="D95" t="inlineStr">
+      <c r="D95" s="5" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at BYJU'S with 5.6 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Weaviate, Pinecone) matching the JD. Platform Signals: Based in Vizag; 60-day notice; active GitHub (score 22).</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" t="inlineStr">
+      <c r="A96" s="7" t="inlineStr">
         <is>
           <t>CAND_0070025</t>
         </is>
       </c>
-      <c r="B96" t="n">
+      <c r="B96" s="8" t="n">
         <v>95</v>
       </c>
-      <c r="C96" t="n">
+      <c r="C96" s="8" t="n">
         <v>0.2304</v>
       </c>
-      <c r="D96" t="inlineStr">
+      <c r="D96" s="7" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Hooli with 5.3 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (GraphQL, BigQuery, FastAPI) matching the JD. Platform Signals: Based in Noida (direct hybrid match); 90-day notice; active GitHub (score 53).</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" t="inlineStr">
+      <c r="A97" s="5" t="inlineStr">
         <is>
           <t>CAND_0013625</t>
         </is>
       </c>
-      <c r="B97" t="n">
+      <c r="B97" s="6" t="n">
         <v>96</v>
       </c>
-      <c r="C97" t="n">
+      <c r="C97" s="6" t="n">
         <v>0.2277</v>
       </c>
-      <c r="D97" t="inlineStr">
+      <c r="D97" s="5" t="inlineStr">
         <is>
           <t>Current Role: Senior Software Engineer at Freshworks with 6.2 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Deep Learning, Time Series, Angular) matching the JD. Platform Signals: Based in Gurgaon; 30-day notice (highly immediate availability); active GitHub (score 25).</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" t="inlineStr">
+      <c r="A98" s="7" t="inlineStr">
         <is>
           <t>CAND_0050876</t>
         </is>
       </c>
-      <c r="B98" t="n">
+      <c r="B98" s="8" t="n">
         <v>97</v>
       </c>
-      <c r="C98" t="n">
+      <c r="C98" s="8" t="n">
         <v>0.2194</v>
       </c>
-      <c r="D98" t="inlineStr">
+      <c r="D98" s="7" t="inlineStr">
         <is>
           <t>Current Role: Applied ML Engineer at Freshworks with 6.0 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Qdrant, FAISS, OpenSearch) matching the JD. Platform Signals: Based in Kolkata; 90-day notice; strong GitHub portfolio (score 86).</t>
         </is>
       </c>
     </row>
     <row r="99">
-      <c r="A99" t="inlineStr">
+      <c r="A99" s="5" t="inlineStr">
         <is>
           <t>CAND_0006766</t>
         </is>
       </c>
-      <c r="B99" t="n">
+      <c r="B99" s="6" t="n">
         <v>98</v>
       </c>
-      <c r="C99" t="n">
+      <c r="C99" s="6" t="n">
         <v>0.2055</v>
       </c>
-      <c r="D99" t="inlineStr">
+      <c r="D99" s="5" t="inlineStr">
         <is>
           <t>Current Role: Senior Software Engineer at PhonePe with 6.4 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (LoRA, Flask, Kafka) matching the JD. Platform Signals: Based in Jaipur; 30-day notice (highly immediate availability); active GitHub (score 57).</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" t="inlineStr">
+      <c r="A100" s="7" t="inlineStr">
         <is>
           <t>CAND_0090178</t>
         </is>
       </c>
-      <c r="B100" t="n">
+      <c r="B100" s="8" t="n">
         <v>99</v>
       </c>
-      <c r="C100" t="n">
+      <c r="C100" s="8" t="n">
         <v>0.2055</v>
       </c>
-      <c r="D100" t="inlineStr">
+      <c r="D100" s="7" t="inlineStr">
         <is>
           <t>Current Role: Data Engineer at PhonePe with 7.1 years of experience. Skill Alignment: Demonstrates strong NLP/Vector search skills (Milvus, Weaviate) matching the JD. Platform Signals: Based in Gurgaon; 90-day notice.</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" t="inlineStr">
+      <c r="A101" s="5" t="inlineStr">
         <is>
           <t>CAND_0093117</t>
         </is>
       </c>
-      <c r="B101" t="n">
+      <c r="B101" s="6" t="n">
         <v>100</v>
       </c>
-      <c r="C101" t="n">
+      <c r="C101" s="6" t="n">
         <v>0.2</v>
       </c>
-      <c r="D101" t="inlineStr">
+      <c r="D101" s="5" t="inlineStr">
         <is>
           <t>Current Role: Software Engineer at Hooli with 5.0 years of experience. Skill Alignment: Demonstrates proficiency in key ML skills (Angular, Rust, GraphQL) matching the JD. Platform Signals: Based in Bangalore (willing to relocate); 60-day notice.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D101"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>